<commit_message>
Fixed bad MPN of the battery's connector.
</commit_message>
<xml_diff>
--- a/Electronics/v7.4/production/BOM.xlsx
+++ b/Electronics/v7.4/production/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\open-ephys\FED3\Electronics\v7.4\production\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\KravitzLabDevices\FED3\Electronics\v7.4\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231CF8E9-F4D9-4E46-910B-9F8B43BCA178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0D4A7C-E796-49CA-97AC-9AA490DEB114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2C14BB60-4DCF-4356-9B2A-66B802743BE9}"/>
+    <workbookView xWindow="-390" yWindow="2985" windowWidth="21600" windowHeight="11295" xr2:uid="{2C14BB60-4DCF-4356-9B2A-66B802743BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -181,9 +181,6 @@
     <t>X5</t>
   </si>
   <si>
-    <t>JST-XH-02</t>
-  </si>
-  <si>
     <t>USB0</t>
   </si>
   <si>
@@ -520,12 +517,6 @@
     <t>CONN MICRO SD CARD R/A</t>
   </si>
   <si>
-    <t>OEPS070028</t>
-  </si>
-  <si>
-    <t>B2B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
     <t>Generic connector, single row, 01x02</t>
   </si>
   <si>
@@ -593,6 +584,15 @@
   </si>
   <si>
     <t>VFHR1116P-4C82A-TR</t>
+  </si>
+  <si>
+    <t>OEPS070130</t>
+  </si>
+  <si>
+    <t>B2B-PH-K-S(LF)(SN)</t>
+  </si>
+  <si>
+    <t>B2B-PH-K-S</t>
   </si>
 </sst>
 </file>
@@ -994,25 +994,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>162</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1029,13 +1029,13 @@
         <v>40</v>
       </c>
       <c r="E2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" t="s">
         <v>63</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>64</v>
-      </c>
-      <c r="G2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1052,13 +1052,13 @@
         <v>13</v>
       </c>
       <c r="E3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" t="s">
         <v>66</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>67</v>
-      </c>
-      <c r="G3" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1066,22 +1066,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>50</v>
-      </c>
       <c r="E4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" t="s">
         <v>69</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>70</v>
-      </c>
-      <c r="G4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1089,7 +1089,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C5" s="1">
         <v>8</v>
@@ -1098,13 +1098,13 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>73</v>
-      </c>
-      <c r="G5" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1112,7 +1112,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C6" s="1">
         <v>2</v>
@@ -1121,13 +1121,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>76</v>
-      </c>
-      <c r="G6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1135,7 +1135,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C7" s="1">
         <v>9</v>
@@ -1144,13 +1144,13 @@
         <v>10</v>
       </c>
       <c r="E7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>79</v>
-      </c>
-      <c r="G7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1158,7 +1158,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C8" s="1">
         <v>2</v>
@@ -1167,13 +1167,13 @@
         <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F8" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="G8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1181,22 +1181,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="G9" t="s">
         <v>82</v>
-      </c>
-      <c r="F9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1213,13 +1213,13 @@
         <v>31</v>
       </c>
       <c r="E10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" t="s">
         <v>84</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>85</v>
-      </c>
-      <c r="G10" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1236,13 +1236,13 @@
         <v>25</v>
       </c>
       <c r="E11" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" t="s">
         <v>87</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>88</v>
-      </c>
-      <c r="G11" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1259,13 +1259,13 @@
         <v>38</v>
       </c>
       <c r="E12" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" t="s">
         <v>90</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>91</v>
-      </c>
-      <c r="G12" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1282,13 +1282,13 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" t="s">
         <v>93</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>94</v>
-      </c>
-      <c r="G13" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1305,13 +1305,13 @@
         <v>16</v>
       </c>
       <c r="E14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" t="s">
         <v>96</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>97</v>
-      </c>
-      <c r="G14" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1319,7 +1319,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C15" s="1">
         <v>3</v>
@@ -1328,13 +1328,13 @@
         <v>14</v>
       </c>
       <c r="E15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1342,22 +1342,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C16" s="1">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" t="s">
         <v>100</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>101</v>
-      </c>
-      <c r="G16" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1365,22 +1365,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="1">
-        <v>1</v>
-      </c>
-      <c r="D17" t="s">
-        <v>52</v>
-      </c>
       <c r="E17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1388,22 +1388,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C18" s="1">
         <v>3</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" t="s">
         <v>104</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>105</v>
-      </c>
-      <c r="G18" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1420,13 +1420,13 @@
         <v>19</v>
       </c>
       <c r="E19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
         <v>19</v>
       </c>
       <c r="G19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1434,22 +1434,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="1">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s">
-        <v>48</v>
-      </c>
       <c r="E20" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" t="s">
         <v>109</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>110</v>
-      </c>
-      <c r="G20" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1466,13 +1466,13 @@
         <v>23</v>
       </c>
       <c r="E21" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" t="s">
         <v>112</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>113</v>
-      </c>
-      <c r="G21" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1489,13 +1489,13 @@
         <v>35</v>
       </c>
       <c r="E22" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" t="s">
         <v>115</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>116</v>
-      </c>
-      <c r="G22" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1503,7 +1503,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C23" s="1">
         <v>5</v>
@@ -1512,13 +1512,13 @@
         <v>6</v>
       </c>
       <c r="E23" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" t="s">
         <v>118</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>119</v>
-      </c>
-      <c r="G23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1526,7 +1526,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C24" s="1">
         <v>3</v>
@@ -1535,13 +1535,13 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" t="s">
         <v>121</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>122</v>
-      </c>
-      <c r="G24" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C25" s="1">
         <v>2</v>
@@ -1558,13 +1558,13 @@
         <v>9</v>
       </c>
       <c r="E25" t="s">
+        <v>123</v>
+      </c>
+      <c r="F25" t="s">
         <v>124</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>125</v>
-      </c>
-      <c r="G25" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1572,7 +1572,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C26" s="1">
         <v>3</v>
@@ -1581,13 +1581,13 @@
         <v>17</v>
       </c>
       <c r="E26" t="s">
+        <v>126</v>
+      </c>
+      <c r="F26" t="s">
         <v>127</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>128</v>
-      </c>
-      <c r="G26" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1604,13 +1604,13 @@
         <v>4</v>
       </c>
       <c r="E27" t="s">
+        <v>129</v>
+      </c>
+      <c r="F27" t="s">
+        <v>175</v>
+      </c>
+      <c r="G27" t="s">
         <v>130</v>
-      </c>
-      <c r="F27" t="s">
-        <v>178</v>
-      </c>
-      <c r="G27" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1618,22 +1618,22 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>131</v>
+      </c>
+      <c r="F28" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="1">
-        <v>1</v>
-      </c>
-      <c r="D28" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="G28" t="s">
         <v>132</v>
-      </c>
-      <c r="F28" t="s">
-        <v>60</v>
-      </c>
-      <c r="G28" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1650,13 +1650,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="s">
+        <v>133</v>
+      </c>
+      <c r="F29" t="s">
         <v>134</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>135</v>
-      </c>
-      <c r="G29" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1673,13 +1673,13 @@
         <v>42</v>
       </c>
       <c r="E30" t="s">
+        <v>136</v>
+      </c>
+      <c r="F30" t="s">
         <v>137</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>138</v>
-      </c>
-      <c r="G30" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1687,22 +1687,22 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="1">
-        <v>1</v>
-      </c>
-      <c r="D31" t="s">
-        <v>57</v>
-      </c>
       <c r="E31" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" t="s">
         <v>140</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>141</v>
-      </c>
-      <c r="G31" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1719,13 +1719,13 @@
         <v>27</v>
       </c>
       <c r="E32" t="s">
+        <v>142</v>
+      </c>
+      <c r="F32" t="s">
         <v>143</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>144</v>
-      </c>
-      <c r="G32" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1733,22 +1733,22 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="1">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" t="s">
-        <v>46</v>
-      </c>
       <c r="E33" t="s">
+        <v>145</v>
+      </c>
+      <c r="F33" t="s">
         <v>146</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>147</v>
-      </c>
-      <c r="G33" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1765,13 +1765,13 @@
         <v>29</v>
       </c>
       <c r="E34" t="s">
+        <v>148</v>
+      </c>
+      <c r="F34" t="s">
         <v>149</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>150</v>
-      </c>
-      <c r="G34" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1788,13 +1788,13 @@
         <v>8</v>
       </c>
       <c r="E35" t="s">
+        <v>151</v>
+      </c>
+      <c r="F35" t="s">
         <v>152</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>153</v>
-      </c>
-      <c r="G35" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1811,13 +1811,13 @@
         <v>33</v>
       </c>
       <c r="E36" t="s">
+        <v>154</v>
+      </c>
+      <c r="F36" t="s">
+        <v>176</v>
+      </c>
+      <c r="G36" t="s">
         <v>155</v>
-      </c>
-      <c r="F36" t="s">
-        <v>179</v>
-      </c>
-      <c r="G36" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1831,16 +1831,16 @@
         <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>44</v>
+        <v>181</v>
       </c>
       <c r="E37" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="F37" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="G37" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>